<commit_message>
updated final project on 12-09-2026
</commit_message>
<xml_diff>
--- a/rasi_modaddress.xlsx
+++ b/rasi_modaddress.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kabish\plc_projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{942502E6-1063-4AC7-B733-04E17CC01A03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFEA3265-70A8-4DB1-91D3-62D7D2F3972B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="16533" xr2:uid="{8C8DA64F-F3DA-4B62-857A-01C3BAFCB6A6}"/>
+    <workbookView xWindow="3330" yWindow="7583" windowWidth="21600" windowHeight="13582" xr2:uid="{8C8DA64F-F3DA-4B62-857A-01C3BAFCB6A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
   <si>
     <t xml:space="preserve"> modbus</t>
   </si>
@@ -131,6 +131,12 @@
   </si>
   <si>
     <t>run</t>
+  </si>
+  <si>
+    <t>Auto_Active_Live_Weight</t>
+  </si>
+  <si>
+    <t>Semi_Auto_Active_Live_Weight</t>
   </si>
 </sst>
 </file>
@@ -490,22 +496,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD4C5175-4C52-4D97-A347-EDAE51E383ED}">
   <dimension ref="B1:O44"/>
-  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="27.3515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.46875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.9375" customWidth="1"/>
-    <col min="6" max="6" width="18.05859375" customWidth="1"/>
-    <col min="7" max="7" width="27.3515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.87890625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.3515625" customWidth="1"/>
-    <col min="10" max="10" width="14.17578125" customWidth="1"/>
-    <col min="12" max="12" width="22.52734375" customWidth="1"/>
-    <col min="13" max="13" width="16.17578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="28.1171875" customWidth="1"/>
+    <col min="2" max="2" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.46484375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.9296875" customWidth="1"/>
+    <col min="6" max="6" width="18.06640625" customWidth="1"/>
+    <col min="7" max="7" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.86328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" customWidth="1"/>
+    <col min="10" max="10" width="14.19921875" customWidth="1"/>
+    <col min="12" max="12" width="22.53125" customWidth="1"/>
+    <col min="13" max="13" width="16.19921875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="28.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="1" spans="2:15" x14ac:dyDescent="0.45">
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
@@ -523,7 +529,7 @@
       </c>
       <c r="J1" s="2"/>
     </row>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.45">
       <c r="C2" t="s">
         <v>0</v>
       </c>
@@ -549,7 +555,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B3">
         <v>1</v>
       </c>
@@ -578,7 +584,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B4">
         <v>2</v>
       </c>
@@ -607,7 +613,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B5">
         <v>3</v>
       </c>
@@ -639,7 +645,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B6">
         <v>4</v>
       </c>
@@ -668,7 +674,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B7">
         <v>5</v>
       </c>
@@ -697,7 +703,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B8">
         <v>6</v>
       </c>
@@ -726,7 +732,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B9">
         <v>7</v>
       </c>
@@ -749,7 +755,7 @@
       </c>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B10">
         <v>8</v>
       </c>
@@ -778,7 +784,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B11">
         <v>9</v>
       </c>
@@ -807,7 +813,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B12">
         <v>10</v>
       </c>
@@ -836,7 +842,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B13">
         <v>11</v>
       </c>
@@ -865,7 +871,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B14">
         <v>12</v>
       </c>
@@ -894,7 +900,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B15">
         <v>13</v>
       </c>
@@ -923,7 +929,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.5">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B16">
         <v>14</v>
       </c>
@@ -952,7 +958,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B17">
         <v>15</v>
       </c>
@@ -981,7 +987,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B18">
         <v>16</v>
       </c>
@@ -1010,7 +1016,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B19">
         <v>17</v>
       </c>
@@ -1039,7 +1045,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B20">
         <v>18</v>
       </c>
@@ -1050,7 +1056,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B21">
         <v>19</v>
       </c>
@@ -1061,7 +1067,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B22">
         <v>20</v>
       </c>
@@ -1072,12 +1078,12 @@
         <v>119</v>
       </c>
     </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="28" spans="2:10" x14ac:dyDescent="0.45">
       <c r="H28" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="29" spans="2:10" x14ac:dyDescent="0.45">
       <c r="C29" t="s">
         <v>11</v>
       </c>
@@ -1091,7 +1097,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="30" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B30" t="s">
         <v>12</v>
       </c>
@@ -1108,7 +1114,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="31" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B31" t="s">
         <v>14</v>
       </c>
@@ -1125,7 +1131,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.5">
+    <row r="32" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B32" t="s">
         <v>15</v>
       </c>
@@ -1142,7 +1148,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.5">
+    <row r="33" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B33" t="s">
         <v>16</v>
       </c>
@@ -1159,7 +1165,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.5">
+    <row r="34" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B34" t="s">
         <v>28</v>
       </c>
@@ -1176,7 +1182,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.5">
+    <row r="35" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B35" t="s">
         <v>31</v>
       </c>
@@ -1193,7 +1199,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.5">
+    <row r="36" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G36" t="s">
         <v>26</v>
       </c>
@@ -1201,7 +1207,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.5">
+    <row r="37" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G37" t="s">
         <v>27</v>
       </c>
@@ -1209,7 +1215,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.5">
+    <row r="39" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B39" t="s">
         <v>24</v>
       </c>
@@ -1220,7 +1226,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.5">
+    <row r="40" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B40" t="s">
         <v>25</v>
       </c>
@@ -1231,7 +1237,10 @@
         <v>342</v>
       </c>
     </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.5">
+    <row r="41" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B41" t="s">
+        <v>32</v>
+      </c>
       <c r="C41">
         <v>172</v>
       </c>
@@ -1239,7 +1248,10 @@
         <v>344</v>
       </c>
     </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.5">
+    <row r="42" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B42" t="s">
+        <v>33</v>
+      </c>
       <c r="C42">
         <v>173</v>
       </c>
@@ -1247,7 +1259,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.5">
+    <row r="43" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B43" t="s">
         <v>29</v>
       </c>
@@ -1258,7 +1270,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.5">
+    <row r="44" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B44" t="s">
         <v>30</v>
       </c>

</xml_diff>